<commit_message>
feat: Finalize project features, fix performance test, and update presentation slides
</commit_message>
<xml_diff>
--- a/SmartShop_TestReport.xlsx
+++ b/SmartShop_TestReport.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="99">
   <si>
     <t>PASS / FAIL</t>
   </si>
   <si>
-    <t>Ngày kiểm thử: 23:30 24/05/2026   |   Tổng: 9 test case   |   Pass: 9   |   Fail: 0</t>
+    <t>Ngày kiểm thử: 00:26 26/06/2026   |   Tổng: 11 test case   |   Pass: 11   |   Fail: 0</t>
   </si>
   <si>
     <t>Mã TC</t>
@@ -71,10 +71,10 @@
     <t>HTTP 200 và access_token hợp lệ</t>
   </si>
   <si>
-    <t>HTTP 201 – 383ms</t>
-  </si>
-  <si>
-    <t>383ms</t>
+    <t>HTTP 201 – 201ms</t>
+  </si>
+  <si>
+    <t>201ms</t>
   </si>
   <si>
     <t>PASS</t>
@@ -98,10 +98,10 @@
     <t>HTTP 200, trả về mảng items và tổng số total</t>
   </si>
   <si>
-    <t>HTTP 200 – 189ms</t>
-  </si>
-  <si>
-    <t>189ms</t>
+    <t>HTTP 200 – 1289ms</t>
+  </si>
+  <si>
+    <t>1289ms</t>
   </si>
   <si>
     <t>UT-03</t>
@@ -119,10 +119,31 @@
     <t>HTTP 200, trả về mảng danh mục không rỗng</t>
   </si>
   <si>
-    <t>HTTP 200 – 12ms</t>
-  </si>
-  <si>
-    <t>12ms</t>
+    <t>HTTP 200 – 104ms</t>
+  </si>
+  <si>
+    <t>104ms</t>
+  </si>
+  <si>
+    <t>UT-04</t>
+  </si>
+  <si>
+    <t>Đăng ký tài khoản mới</t>
+  </si>
+  <si>
+    <t>Đăng ký người dùng (Register)</t>
+  </si>
+  <si>
+    <t>http://localhost:3001/api/auth/register</t>
+  </si>
+  <si>
+    <t>HTTP 201 và tạo thành công</t>
+  </si>
+  <si>
+    <t>HTTP 201 – 279ms</t>
+  </si>
+  <si>
+    <t>279ms</t>
   </si>
   <si>
     <t>IT-01</t>
@@ -143,10 +164,10 @@
     <t>HTTP 200, trả về thông tin user với email và role chính xác</t>
   </si>
   <si>
-    <t>HTTP 200 – 10ms</t>
-  </si>
-  <si>
-    <t>10ms</t>
+    <t>HTTP 200 – 150ms</t>
+  </si>
+  <si>
+    <t>150ms</t>
   </si>
   <si>
     <t>IT-02</t>
@@ -164,10 +185,10 @@
     <t>HTTP 200, danh sách sản phẩm lọc đúng theo categoryId=1</t>
   </si>
   <si>
-    <t>HTTP 200 – 19ms</t>
-  </si>
-  <si>
-    <t>19ms</t>
+    <t>HTTP 200 – 102ms</t>
+  </si>
+  <si>
+    <t>102ms</t>
   </si>
   <si>
     <t>IT-03</t>
@@ -185,10 +206,31 @@
     <t>HTTP 200 nếu mã hợp lệ; HTTP 404 nếu mã không tồn tại</t>
   </si>
   <si>
-    <t>HTTP 200 – 9ms</t>
-  </si>
-  <si>
-    <t>9ms</t>
+    <t>HTTP 200 – 100ms</t>
+  </si>
+  <si>
+    <t>100ms</t>
+  </si>
+  <si>
+    <t>IT-04</t>
+  </si>
+  <si>
+    <t>Giỏ hàng và Checkout (Cart)</t>
+  </si>
+  <si>
+    <t>Tích hợp Giỏ hàng và Thanh toán</t>
+  </si>
+  <si>
+    <t>http://localhost:3001/api/orders</t>
+  </si>
+  <si>
+    <t>HTTP 201, tạo đơn hàng thành công</t>
+  </si>
+  <si>
+    <t>HTTP 201 – 1244ms</t>
+  </si>
+  <si>
+    <t>1244ms</t>
   </si>
   <si>
     <t>ST-01</t>
@@ -203,16 +245,13 @@
     <t>Đặt hàng không cần đăng nhập (Guest Checkout)</t>
   </si>
   <si>
-    <t>http://localhost:3001/api/orders</t>
-  </si>
-  <si>
     <t>HTTP 201, tạo đơn hàng mới với status PENDING</t>
   </si>
   <si>
-    <t>HTTP 201 – 168ms</t>
-  </si>
-  <si>
-    <t>168ms</t>
+    <t>HTTP 201 – 729ms</t>
+  </si>
+  <si>
+    <t>729ms</t>
   </si>
   <si>
     <t>ST-02</t>
@@ -230,10 +269,10 @@
     <t>HTTP 200, trả về totalRevenue, totalOrders, totalProducts, totalUsers</t>
   </si>
   <si>
-    <t>HTTP 200 – 77ms</t>
-  </si>
-  <si>
-    <t>77ms</t>
+    <t>HTTP 200 – 627ms</t>
+  </si>
+  <si>
+    <t>627ms</t>
   </si>
   <si>
     <t>ST-03</t>
@@ -251,10 +290,10 @@
     <t>HTTP 200, AI trả về câu trả lời không rỗng</t>
   </si>
   <si>
-    <t>HTTP 201 – 30510ms</t>
-  </si>
-  <si>
-    <t>30510ms</t>
+    <t>HTTP 201 – 20564ms</t>
+  </si>
+  <si>
+    <t>20564ms</t>
   </si>
   <si>
     <t>BẢNG TỔNG KẾT KIỂM THỬ</t>
@@ -821,7 +860,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1006,35 +1045,35 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="5">
+        <v>201</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="I7" s="8">
-        <v>200</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>21</v>
@@ -1042,13 +1081,13 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>39</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>47</v>
@@ -1083,7 +1122,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>54</v>
@@ -1111,70 +1150,70 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="E10" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="10" t="s">
+      <c r="G10" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="I10" s="8">
+        <v>200</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="I10" s="10">
-        <v>201</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>66</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="G11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="8">
+        <v>201</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="I11" s="10">
-        <v>200</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>21</v>
@@ -1182,13 +1221,13 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>61</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>76</v>
@@ -1197,21 +1236,91 @@
         <v>16</v>
       </c>
       <c r="F12" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="H12" s="10" t="s">
         <v>78</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>79</v>
       </c>
       <c r="I12" s="10">
         <v>201</v>
       </c>
       <c r="J12" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="B13" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I13" s="10">
+        <v>200</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I14" s="10">
+        <v>201</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K14" s="6" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1236,7 +1345,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1247,13 +1356,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1261,10 +1370,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" s="13">
         <v>0</v>
@@ -1272,13 +1381,13 @@
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B4" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="13">
         <v>0</v>
@@ -1286,7 +1395,7 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B5" s="13">
         <v>3</v>
@@ -1300,13 +1409,13 @@
     </row>
     <row r="6" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="B6" s="14">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6" s="14">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D6" s="14">
         <v>0</v>

</xml_diff>

<commit_message>
Fix: Bỏ cờ accept-data-loss nguy hiểm khi deploy
</commit_message>
<xml_diff>
--- a/SmartShop_TestReport.xlsx
+++ b/SmartShop_TestReport.xlsx
@@ -17,7 +17,7 @@
     <t>PASS / FAIL</t>
   </si>
   <si>
-    <t>Ngày kiểm thử: 00:26 26/06/2026   |   Tổng: 11 test case   |   Pass: 11   |   Fail: 0</t>
+    <t>Ngày kiểm thử: 09:19 27/06/2026   |   Tổng: 11 test case   |   Pass: 11   |   Fail: 0</t>
   </si>
   <si>
     <t>Mã TC</t>
@@ -71,10 +71,10 @@
     <t>HTTP 200 và access_token hợp lệ</t>
   </si>
   <si>
-    <t>HTTP 201 – 201ms</t>
-  </si>
-  <si>
-    <t>201ms</t>
+    <t>HTTP 201 – 314ms</t>
+  </si>
+  <si>
+    <t>314ms</t>
   </si>
   <si>
     <t>PASS</t>
@@ -98,10 +98,10 @@
     <t>HTTP 200, trả về mảng items và tổng số total</t>
   </si>
   <si>
-    <t>HTTP 200 – 1289ms</t>
-  </si>
-  <si>
-    <t>1289ms</t>
+    <t>HTTP 200 – 605ms</t>
+  </si>
+  <si>
+    <t>605ms</t>
   </si>
   <si>
     <t>UT-03</t>
@@ -119,10 +119,10 @@
     <t>HTTP 200, trả về mảng danh mục không rỗng</t>
   </si>
   <si>
-    <t>HTTP 200 – 104ms</t>
-  </si>
-  <si>
-    <t>104ms</t>
+    <t>HTTP 200 – 131ms</t>
+  </si>
+  <si>
+    <t>131ms</t>
   </si>
   <si>
     <t>UT-04</t>
@@ -140,10 +140,10 @@
     <t>HTTP 201 và tạo thành công</t>
   </si>
   <si>
-    <t>HTTP 201 – 279ms</t>
-  </si>
-  <si>
-    <t>279ms</t>
+    <t>HTTP 201 – 288ms</t>
+  </si>
+  <si>
+    <t>288ms</t>
   </si>
   <si>
     <t>IT-01</t>
@@ -164,10 +164,10 @@
     <t>HTTP 200, trả về thông tin user với email và role chính xác</t>
   </si>
   <si>
-    <t>HTTP 200 – 150ms</t>
-  </si>
-  <si>
-    <t>150ms</t>
+    <t>HTTP 200 – 165ms</t>
+  </si>
+  <si>
+    <t>165ms</t>
   </si>
   <si>
     <t>IT-02</t>
@@ -185,10 +185,10 @@
     <t>HTTP 200, danh sách sản phẩm lọc đúng theo categoryId=1</t>
   </si>
   <si>
-    <t>HTTP 200 – 102ms</t>
-  </si>
-  <si>
-    <t>102ms</t>
+    <t>HTTP 200 – 116ms</t>
+  </si>
+  <si>
+    <t>116ms</t>
   </si>
   <si>
     <t>IT-03</t>
@@ -206,10 +206,10 @@
     <t>HTTP 200 nếu mã hợp lệ; HTTP 404 nếu mã không tồn tại</t>
   </si>
   <si>
-    <t>HTTP 200 – 100ms</t>
-  </si>
-  <si>
-    <t>100ms</t>
+    <t>HTTP 200 – 110ms</t>
+  </si>
+  <si>
+    <t>110ms</t>
   </si>
   <si>
     <t>IT-04</t>
@@ -227,10 +227,10 @@
     <t>HTTP 201, tạo đơn hàng thành công</t>
   </si>
   <si>
-    <t>HTTP 201 – 1244ms</t>
-  </si>
-  <si>
-    <t>1244ms</t>
+    <t>HTTP 201 – 1262ms</t>
+  </si>
+  <si>
+    <t>1262ms</t>
   </si>
   <si>
     <t>ST-01</t>
@@ -248,10 +248,10 @@
     <t>HTTP 201, tạo đơn hàng mới với status PENDING</t>
   </si>
   <si>
-    <t>HTTP 201 – 729ms</t>
-  </si>
-  <si>
-    <t>729ms</t>
+    <t>HTTP 201 – 728ms</t>
+  </si>
+  <si>
+    <t>728ms</t>
   </si>
   <si>
     <t>ST-02</t>
@@ -269,10 +269,10 @@
     <t>HTTP 200, trả về totalRevenue, totalOrders, totalProducts, totalUsers</t>
   </si>
   <si>
-    <t>HTTP 200 – 627ms</t>
-  </si>
-  <si>
-    <t>627ms</t>
+    <t>HTTP 200 – 732ms</t>
+  </si>
+  <si>
+    <t>732ms</t>
   </si>
   <si>
     <t>ST-03</t>
@@ -290,10 +290,10 @@
     <t>HTTP 200, AI trả về câu trả lời không rỗng</t>
   </si>
   <si>
-    <t>HTTP 201 – 20564ms</t>
-  </si>
-  <si>
-    <t>20564ms</t>
+    <t>HTTP 201 – 49701ms</t>
+  </si>
+  <si>
+    <t>49701ms</t>
   </si>
   <si>
     <t>BẢNG TỔNG KẾT KIỂM THỬ</t>

</xml_diff>